<commit_message>
Ajuste na seleção de comprador (SUPPLY) no robô GAM Supply
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_entrada/mix.xlsx
+++ b/Aplicativos/GAM/bd_entrada/mix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alessandro.soares.BAKLIZI\Downloads\Equipes_Agentes\Aplicativos\GAM\bd_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C76BE1-AAB4-4D40-8C4E-C9AB2CD658C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0860F2-2D46-4690-9730-4B21CBC7896E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$55</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="65">
   <si>
     <t>Código Empresa</t>
   </si>
@@ -57,14 +57,179 @@
     <t>A</t>
   </si>
   <si>
-    <t>desativar outra hora</t>
+    <t>REFRE FRUKITO PET 500ML UVA</t>
+  </si>
+  <si>
+    <t>REFRIG COLA FRUKI PET 600ML COLA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI CITRUS LT 350ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFRIG FRUKI COLA LT 350ML </t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI COLA PET 200ML COLA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI FRAMB PET 2L</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI FRAMBOESA PET 200ML FRAMBOESA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUAR LT 350ML C BERGA ZR</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUAR ZR PET 3L GUARANA ZERO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUARAN C ABAC LT 350ML GUARANA ABACAX</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUARAN LT 350ML GUARA C BERGA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUARAN LT 350ML GUARANA ZERO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUARANA LIGHT ZERO PET 600M</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUARANA LT 350ML GUARANA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUARANA PET 200ML GUARANA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUARANA ZR PET 2L GUARANA ZERO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI LAB PASSION LT 350ML</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI LARANJA LT 350ML LARANJA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI LT 269ML GUARANA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI LT 350 ML COLA ZR</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI LT 350ML LIMAO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 1 5 L CITRUS</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 1 5L GUARANA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 1 5L GUARANA ZERO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 2 L GUARANA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 200 ML GUARANA ZERO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 200ML LARANJA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 200ML LARANJINHA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 200ML LIMAO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 200ML UVA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 2L LARANJA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 2L LARANJINHA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 2L LIMAO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 2L UVA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 3 L LARANJA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 3L GUARANA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 600ML GUARANA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 600ML LARANJA</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 600ML LIMAO</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI UVA PET 600ML UVA</t>
+  </si>
+  <si>
+    <t>REFRIG GUARANA FRUKI PET 600ML ZERO</t>
+  </si>
+  <si>
+    <t>REFRIGC COLA FRUKI PET 2 L COLA</t>
+  </si>
+  <si>
+    <t>REFRIGC COLA FRUKI PET 2 L COLA ZERO</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM LARANJA VD 1L</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM TP 1L LARANJA</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM TP 1L MACA</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM TP 1L UVA</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM TP 200ML LARANJA</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM TP 200ML MACA</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM TP 200ML UVA E MACA</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM UVA VD 1L</t>
+  </si>
+  <si>
+    <t>SUCO COM TEM VERDE VD 1L</t>
+  </si>
+  <si>
+    <t>VH MIORANZA FRISANTE 750ML BCO SV</t>
+  </si>
+  <si>
+    <t>VH MIORANZA FRISANTE 750ML ROSE SV</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>I</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,16 +237,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -89,15 +267,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -379,7 +576,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="75.85546875" bestFit="1" customWidth="1"/>
@@ -417,77 +614,763 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3">
+        <v>376</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3">
+        <v>854</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3">
+        <v>885</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3">
+        <v>877</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="3">
+        <v>767</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="3">
+        <v>35228</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C2">
-        <v>2210</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="C8" s="3">
+        <v>33249</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="3">
+        <v>878</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>15</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="5">
+        <v>33265</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3">
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="3">
+        <v>873</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="3">
+        <v>880</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>15</v>
       </c>
-      <c r="C3">
-        <v>2388</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="B13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="5">
+        <v>882</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4">
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="3">
+        <v>32110</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>15</v>
       </c>
-      <c r="C4">
-        <v>2454</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="B15" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="5">
+        <v>881</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5">
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>15</v>
       </c>
-      <c r="C5">
-        <v>2765</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="B16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="5">
+        <v>769</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>15</v>
       </c>
-      <c r="C6">
-        <v>2785</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="B17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="5">
+        <v>817</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F6" t="s">
-        <v>9</v>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="3">
+        <v>37304</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="3">
+        <v>883</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="3">
+        <v>22871</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="3">
+        <v>875</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="3">
+        <v>884</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="3">
+        <v>742</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>15</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" s="5">
+        <v>743</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="3">
+        <v>744</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>15</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="5">
+        <v>815</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>15</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="5">
+        <v>768</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="3">
+        <v>770</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="3">
+        <v>772</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="3">
+        <v>773</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="3">
+        <v>774</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="3">
+        <v>818</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="3">
+        <v>820</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="3">
+        <v>821</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="3">
+        <v>823</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>15</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C36" s="5">
+        <v>33266</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>15</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C37" s="5">
+        <v>838</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="3">
+        <v>855</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C39" s="3">
+        <v>856</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C40" s="3">
+        <v>857</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C41" s="3">
+        <v>858</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C42" s="3">
+        <v>35225</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C43" s="3">
+        <v>813</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C44" s="3">
+        <v>814</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>63</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C45" s="3">
+        <v>595</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>63</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C46" s="3">
+        <v>582</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>63</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C47" s="3">
+        <v>583</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C48" s="3">
+        <v>584</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>63</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C49" s="3">
+        <v>589</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>63</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50" s="3">
+        <v>590</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>63</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="3">
+        <v>592</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>63</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="3">
+        <v>596</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>63</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C53" s="3">
+        <v>586</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>63</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C54" s="3">
+        <v>33785</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>63</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C55" s="3">
+        <v>33787</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:D55" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D73">
       <sortCondition ref="C1"/>
     </sortState>

</xml_diff>

<commit_message>
Otimização de velocidade de digitação e visão no robô GAM Mix
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_entrada/mix.xlsx
+++ b/Aplicativos/GAM/bd_entrada/mix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alessandro.soares.BAKLIZI\Downloads\Equipes_Agentes\Aplicativos\GAM\bd_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0860F2-2D46-4690-9730-4B21CBC7896E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C546C17D-D78D-49BB-8F9D-D6A469BD5D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$35</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,10 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="65">
-  <si>
-    <t>Código Empresa</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="45">
   <si>
     <t>Empresa : Produto</t>
   </si>
@@ -57,66 +54,6 @@
     <t>A</t>
   </si>
   <si>
-    <t>REFRE FRUKITO PET 500ML UVA</t>
-  </si>
-  <si>
-    <t>REFRIG COLA FRUKI PET 600ML COLA</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI CITRUS LT 350ML</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REFRIG FRUKI COLA LT 350ML </t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI COLA PET 200ML COLA</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI FRAMB PET 2L</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI FRAMBOESA PET 200ML FRAMBOESA</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUAR LT 350ML C BERGA ZR</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUAR ZR PET 3L GUARANA ZERO</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUARAN C ABAC LT 350ML GUARANA ABACAX</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUARAN LT 350ML GUARA C BERGA</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUARAN LT 350ML GUARANA ZERO</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUARANA LIGHT ZERO PET 600M</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUARANA LT 350ML GUARANA</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUARANA PET 200ML GUARANA</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI GUARANA ZR PET 2L GUARANA ZERO</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI LAB PASSION LT 350ML</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI LARANJA LT 350ML LARANJA</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI LT 269ML GUARANA</t>
-  </si>
-  <si>
-    <t>REFRIG FRUKI LT 350 ML COLA ZR</t>
-  </si>
-  <si>
     <t>REFRIG FRUKI LT 350ML LIMAO</t>
   </si>
   <si>
@@ -223,6 +160,9 @@
   </si>
   <si>
     <t>I</t>
+  </si>
+  <si>
+    <t>Código Empresa885</t>
   </si>
 </sst>
 </file>
@@ -576,7 +516,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="75.85546875" bestFit="1" customWidth="1"/>
@@ -589,224 +529,224 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C2" s="3">
-        <v>376</v>
+        <v>884</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3">
+        <v>742</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>15</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3">
-        <v>854</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="3">
-        <v>885</v>
+      <c r="C4" s="5">
+        <v>743</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3">
+        <v>744</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>15</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="3">
-        <v>877</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="5">
+        <v>815</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="3">
-        <v>767</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="3">
-        <v>35228</v>
+      <c r="C7" s="5">
+        <v>768</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3">
-        <v>33249</v>
+        <v>770</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3">
+        <v>772</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="3">
-        <v>878</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>15</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="5">
-        <v>33265</v>
+      <c r="C10" s="3">
+        <v>773</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C11" s="3">
-        <v>873</v>
+        <v>774</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="3">
+        <v>818</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="3">
-        <v>880</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>15</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="5">
-        <v>882</v>
+      <c r="C13" s="3">
+        <v>820</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="3">
+        <v>821</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="3">
-        <v>32110</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>15</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="5">
-        <v>881</v>
+      <c r="C15" s="3">
+        <v>823</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -814,13 +754,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16" s="5">
-        <v>769</v>
+        <v>33266</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -828,550 +768,270 @@
         <v>15</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C17" s="5">
-        <v>817</v>
+        <v>838</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" s="3">
-        <v>37304</v>
+        <v>855</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" s="3">
-        <v>883</v>
+        <v>856</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C20" s="3">
-        <v>22871</v>
+        <v>857</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="3">
-        <v>875</v>
+        <v>858</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C22" s="3">
-        <v>884</v>
+        <v>35225</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="3">
+        <v>813</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="3">
-        <v>742</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>15</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C24" s="5">
-        <v>743</v>
+      <c r="C24" s="3">
+        <v>814</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="3">
+        <v>595</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="3">
-        <v>744</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>15</v>
-      </c>
-      <c r="B26" s="4" t="s">
+      <c r="C26" s="3">
+        <v>582</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C26" s="5">
-        <v>815</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>15</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C27" s="5">
-        <v>768</v>
+      <c r="C27" s="3">
+        <v>583</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C28" s="3">
-        <v>770</v>
+        <v>584</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C29" s="3">
-        <v>772</v>
+        <v>589</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C30" s="3">
-        <v>773</v>
+        <v>590</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C31" s="3">
-        <v>774</v>
+        <v>592</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C32" s="3">
-        <v>818</v>
+        <v>596</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C33" s="3">
-        <v>820</v>
+        <v>586</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C34" s="3">
-        <v>821</v>
+        <v>33785</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C35" s="3">
-        <v>823</v>
+        <v>33787</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>15</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C36" s="5">
-        <v>33266</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>15</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C37" s="5">
-        <v>838</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>63</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C38" s="3">
-        <v>855</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C39" s="3">
-        <v>856</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>63</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C40" s="3">
-        <v>857</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>63</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C41" s="3">
-        <v>858</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>63</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C42" s="3">
-        <v>35225</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>63</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C43" s="3">
-        <v>813</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>63</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C44" s="3">
-        <v>814</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>63</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C45" s="3">
-        <v>595</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C46" s="3">
-        <v>582</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>63</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C47" s="3">
-        <v>583</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>63</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C48" s="3">
-        <v>584</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C49" s="3">
-        <v>589</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>63</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C50" s="3">
-        <v>590</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>63</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C51" s="3">
-        <v>592</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>63</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C52" s="3">
-        <v>596</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>63</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C53" s="3">
-        <v>586</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>63</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C54" s="3">
-        <v>33785</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>63</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C55" s="3">
-        <v>33787</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D55" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D73">
+  <autoFilter ref="A1:D35" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D53">
       <sortCondition ref="C1"/>
     </sortState>
   </autoFilter>

</xml_diff>

<commit_message>
docs: atualização do eco sistema - otimizações ruptura e GAM
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_entrada/mix.xlsx
+++ b/Aplicativos/GAM/bd_entrada/mix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alessandro.soares.BAKLIZI\Downloads\Equipes_Agentes\Aplicativos\GAM\bd_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C546C17D-D78D-49BB-8F9D-D6A469BD5D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{136CFEE3-F7FF-4BDD-AE0A-1415C9B6E0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60" yWindow="3120" windowWidth="28740" windowHeight="10770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -162,7 +162,7 @@
     <t>I</t>
   </si>
   <si>
-    <t>Código Empresa885</t>
+    <t>Código Empresa</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat(GAM/Ruptura): excel exports for buyers and mix grouping optimizations
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_entrada/mix.xlsx
+++ b/Aplicativos/GAM/bd_entrada/mix.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr codeName="EstaPastaDeTrabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alessandro.soares.BAKLIZI\Downloads\Equipes_Agentes\Aplicativos\GAM\bd_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{284DFE32-47CF-4CEA-81BC-CA36AC69A2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068D8F8E-4A59-4CD5-AB6D-15AAA1E3F03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="3120" windowWidth="28740" windowHeight="10770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="glosario" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">glosario!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t>Empresa : Produto</t>
   </si>
@@ -52,6 +53,42 @@
   </si>
   <si>
     <t>Código Empresa</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>TA</t>
+  </si>
+  <si>
+    <t>TIP</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>TIM</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>descrição produto x (loja 1 vai estar ativo)</t>
+  </si>
+  <si>
+    <t>descrição produto x (para todas as lojas vai estar ativo, Exceto loja 1)</t>
+  </si>
+  <si>
+    <t>descrição produto x (exeto lojas pequenas, fica ativo para outras menos pra as pequenas)</t>
+  </si>
+  <si>
+    <t>descrição produto x (exeto lojas pequenas e Médias, fica ativo só para as grandes)</t>
+  </si>
+  <si>
+    <t>I</t>
   </si>
 </sst>
 </file>
@@ -373,12 +410,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="75.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="81.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="30.42578125" bestFit="1" customWidth="1"/>
@@ -410,13 +448,121 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>411</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D19">
-      <sortCondition ref="C1"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F70CD23-A5D7-45F5-AD31-9A2F66EEC663}">
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="81.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <v>1234</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3">
+        <v>456</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4">
+        <v>87987</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5">
+        <v>4564</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: initialize virtual environment dependencies and add agent skill documentation
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_entrada/mix.xlsx
+++ b/Aplicativos/GAM/bd_entrada/mix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alessandro.soares.BAKLIZI\Downloads\Equipes_Agentes\Aplicativos\GAM\bd_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068D8F8E-4A59-4CD5-AB6D-15AAA1E3F03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DAF68A5-BEA9-411D-A261-FDD3287ECFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
   <si>
     <t>Empresa : Produto</t>
   </si>
@@ -86,9 +86,6 @@
   </si>
   <si>
     <t>descrição produto x (exeto lojas pequenas e Médias, fica ativo só para as grandes)</t>
-  </si>
-  <si>
-    <t>I</t>
   </si>
 </sst>
 </file>
@@ -410,7 +407,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -446,17 +443,6 @@
       </c>
       <c r="I1" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>411</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(ruptura): Corrige conversao matematica de float com PyArrow nos dashboards e atualiza regra estrutural Anti-Ponto da base Parquet
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_entrada/mix.xlsx
+++ b/Aplicativos/GAM/bd_entrada/mix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alessandro.soares.BAKLIZI\Downloads\Equipes_Agentes\Aplicativos\GAM\bd_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ADD89BB-B3BE-48FE-9F54-843DEF6C42EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96008300-0EC6-49A8-B222-7E638A295933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6218" uniqueCount="2075">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6226" uniqueCount="2075">
   <si>
     <t>Empresa : Produto</t>
   </si>
@@ -35512,7 +35512,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1CB4010-89E0-4ED5-86E4-002828E0C4B5}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -35623,8 +35623,96 @@
         <v>13</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="C10">
+        <v>36313</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>2704</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3688</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>7841</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>15667</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>7740</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>8213</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>36075</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C9">
+  <conditionalFormatting sqref="C2:C17">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>